<commit_message>
Verify 112-row paging and refine ten-result chat and Excel output
Preserve separate source-date columns, compact private workbooks, publication-safe runtime evidence and explicit narrow-pane and Teams limitations.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agent/exports/template/CorpNetSearchResults.template.xlsx
+++ b/agent/exports/template/CorpNetSearchResults.template.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Results'!$1:$8</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Results'!$A$1:$G$9</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Results'!$A$1:$H$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=";;;&quot;Open file&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,7 +40,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="23"/>
+      <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -67,13 +67,8 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="0025364B"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <color rgb="000563C1"/>
-      <sz val="11"/>
+      <sz val="10"/>
       <u val="single"/>
     </font>
     <font>
@@ -134,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -161,16 +156,19 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -268,14 +266,19 @@
         <t>Open file links to the original. The full URL remains in the cell value; SourceSite is preserved in hidden column F.</t>
       </text>
     </comment>
+    <comment ref="H8" authorId="0" shapeId="0">
+      <text>
+        <t>Source File.TimeCreated in UTC, not export or site-collection creation time. Blank means the source did not supply it.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SearchResults" displayName="SearchResults" ref="A8:G9" headerRowCount="1">
-  <autoFilter ref="A8:G9"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SearchResults" displayName="SearchResults" ref="A8:H9" headerRowCount="1">
+  <autoFilter ref="A8:H9"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Title"/>
     <tableColumn id="2" name="Department"/>
     <tableColumn id="3" name="Tags"/>
@@ -283,6 +286,7 @@
     <tableColumn id="5" name="ModifiedUTC"/>
     <tableColumn id="6" name="SourceSite"/>
     <tableColumn id="7" name="URL"/>
+    <tableColumn id="8" name="CreatedUTC"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -577,19 +581,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col hidden="1" width="38" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" style="1" min="7" max="7"/>
+    <col width="12" customWidth="1" style="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>CorpNet Search Results</t>
@@ -601,8 +606,9 @@
       <c r="E1" s="3" t="n"/>
       <c r="F1" s="3" t="n"/>
       <c r="G1" s="3" t="n"/>
-    </row>
-    <row r="2" ht="34" customHeight="1">
+      <c r="H1" s="3" t="n"/>
+    </row>
+    <row r="2" ht="2" customHeight="1">
       <c r="A2" s="3" t="n"/>
       <c r="B2" s="3" t="n"/>
       <c r="C2" s="3" t="n"/>
@@ -610,8 +616,9 @@
       <c r="E2" s="3" t="n"/>
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="26" customHeight="1">
+      <c r="H2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>SEARCH EXPORT</t>
@@ -623,8 +630,9 @@
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="34" customHeight="1">
+      <c r="H3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
           <t>SCOPE</t>
@@ -640,8 +648,9 @@
       <c r="E4" s="7" t="n"/>
       <c r="F4" s="7" t="n"/>
       <c r="G4" s="7" t="n"/>
-    </row>
-    <row r="5" ht="30" customHeight="1">
+      <c r="H4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>STATUS</t>
@@ -657,8 +666,9 @@
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="7" t="n"/>
       <c r="G5" s="7" t="n"/>
-    </row>
-    <row r="6" ht="32" customHeight="1">
+      <c r="H5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Use the header filters to narrow results. Select Open file to view the original. Full export details: ExportInfo tab.</t>
@@ -670,8 +680,9 @@
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="7" t="n"/>
       <c r="G6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="9" customHeight="1">
+      <c r="H6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="3" customHeight="1">
       <c r="A7" s="7" t="n"/>
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="n"/>
@@ -679,8 +690,9 @@
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
-    </row>
-    <row r="8" ht="28" customHeight="1">
+      <c r="H7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
         <is>
           <t>Title</t>
@@ -716,23 +728,29 @@
           <t>URL</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>CreatedUTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="10" t="n"/>
-      <c r="B9" s="10" t="n"/>
+      <c r="B9" s="11" t="n"/>
       <c r="C9" s="10" t="n"/>
-      <c r="D9" s="10" t="n"/>
-      <c r="E9" s="10" t="n"/>
-      <c r="F9" s="10" t="n"/>
-      <c r="G9" s="11" t="n"/>
+      <c r="D9" s="11" t="n"/>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:G2"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A6:G6"/>
-    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="A6:H6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
@@ -766,128 +784,128 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="13" t="inlineStr">
         <is>
           <t>CorpNet Search Results</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="13" t="inlineStr">
         <is>
           <t>Private, permission-checked search export</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Query</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
       </c>
-      <c r="B3" s="14" t="n"/>
+      <c r="B3" s="15" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>RequestedBy</t>
         </is>
       </c>
-      <c r="B4" s="14" t="n"/>
+      <c r="B4" s="15" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>GeneratedUTC</t>
         </is>
       </c>
-      <c r="B5" s="14" t="n"/>
+      <c r="B5" s="15" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>CompletionStatus</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>TEMPLATE - no search or export has run</t>
         </is>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>CountSemantics</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>The delivery message must distinguish estimated index matches from rows actually exported and disclose any limit, omission or incomplete batch.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Sharing</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>Create a separate workbook per request. Restrict access to the verified requesting user; do not use anonymous or organization-wide links.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>Snapshot</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>The report reflects export time. Original file links remain subject to current SharePoint permissions.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Tags</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Tags are stored source values. Use Excel Text Filters &gt; Contains to filter a tag within a semicolon-delimited value.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="57" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>TemplateInstructions</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Native AddRow writers must insert results before removing the blank placeholder so the new rows inherit body formatting, not the header. Update the table range and set real cell hyperlinks. Do not email this blank template as a completed report.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="57" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>TextSafety</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Treat source titles, tags and other text as literal data, never executable formulas. Text formatting alone is not proof that a particular writer prevents formula injection.</t>
         </is>

</xml_diff>